<commit_message>
Fix PDF download button functionality and append newly crawled startup data
</commit_message>
<xml_diff>
--- a/agtech_startups.xlsx
+++ b/agtech_startups.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -584,6 +584,405 @@
       <c r="K3" t="inlineStr">
         <is>
           <t>2026-06-22 09:26:25</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Vivici</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Not Mentioned</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>FoodTech</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Vivici is a startup focused on scaling the production of precision-fermented dairy proteins.</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>$14.4m</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Grant</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Funding</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxPbGwxM1pDLV9nd1hFQ2FWV0xmRERIcVZDQ0x5dHRhd29qWGd1TFh1Szd0V0s5aVpQVDgxMHdQNmVYSGVEZktZS3pCQTlCU1cyUUswQy1TYllwejdzeFRScGpxeTRNc0ptc0kwRlh4cE80YTJFTWFyWUVodlI5LXlGbUFPMzRxemo0SmVZekNpWGs2Rk1qaXhOVzZqZkNRdXRn?oc=5</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Vivici secured $14.4 million in EIC funding to scale its operations for precision-fermented dairy proteins.</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>2026-06-22 14:29:26</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Rainbow Crops</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Not Mentioned</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Rainbow Crops utilizes AI-powered gene editing technology to develop and advance improved crop varieties.</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>€9.7 million</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Funding</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxPWGxxWFN5aFF1ZWYzc09XUFhPd0xnS21zZl9kWDBSdElXV3hJaWNnano2UVlNSVQ4X00zVWlmczlxdEtsLUZFVUp3LUNfbzBpdXdzY0lsRHN1eXliVTc4bXQzM1BTalVsS2pkMVFJNE9kWUxqNkNMZTVCRGl0SDl5M0VSZExXZnI2b3NJeE5HekViZVplRWplS2pVMzlzbDdUVWZtRnVkbDNVclVWN3V2UVpEdHVoMzI5ODIzUWd6dkNOUW1OODhiMWd6UzlUM2NVcGhCdQ?oc=5</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Rainbow Crops secured €9.7 million in funding to advance its AI-powered gene editing technology for crop improvement.</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>2026-06-22 14:29:43</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Greenda</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Not Mentioned</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Greenda is an AgTech startup that leverages AI to transform traditional field notes into actionable field intelligence for everyday farming operations.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxPUVFJejlsUGNhUi1veW1pTzZSNFJmelNvbHk3cmVtTkJlb09jcC15eW9WTlh4UU5rZWJXSS01M0IwSGpYSjhxVXRoR0pYek1hMlVNdU5rX3JmcnRpeEllQkFGZHROQnhNcVhOVVhCd3oyN3dXU2RmRERJb1hOWGtsd2JGMFRJNGlmaGhEeUxDbFN4eHBjVF9yNFR2Y0VQM3hTSDVZT3FXNHp4SDRIZjRMc0JKWkt1X2xpVF9KSXlB?oc=5</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Greenda is in the news for its AI-driven approach to converting field notes into valuable intelligence for farmers, as highlighted in a sponsored article by EU-Startups.</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>2026-06-22 14:31:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Picketa Systems</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Not Mentioned</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Picketa Systems develops technology to bring crop nutrient testing directly to the field, providing farmers with immediate insights into their crops' health.</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>$1.5m</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Funding</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxOUl9TZTVhNVNHZTFMM3ZCRUVkTjNjeldIaFlvVFRHcmNVQ2lPTTkzUFlHSHA0a3B2ZEwtZjBqUTdxdnZUanhOSHdLeGY3OENlNktDa2RNa3VPc1FLV00tWndaYURFRmxvZnc2TXN3a29sZkYtQWNnS0dDbzAwN1lnSy1jWUtWOWdmYnBVdTdndl91Zw?oc=5</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Picketa Systems has raised $1.5 million to further develop and deploy its in-field crop nutrient testing solutions.</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>2026-06-22 14:32:16</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>OneSoil</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Not Mentioned</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>OneSoil offers an AI Agronomist tool designed to transform fragmented farm data into actionable advice for farmers, aiding in decision-making.</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxONXR5WVNLWGowX2xONVFDaXVPVTUyem1HZkxHTGdNb21jeFlmZHF6WmpDVVI0TUthUmM4RUJQcVBmSkRHRjVZRzBVZnlKNGgxYXRmakhiNVFVN19pN21PMkdVZ1VkVWlRSEZidEIwV0xTMV9uVmZJYzBWQVBVV1h1VzRjYUtBUFg4WWpBeGJVSVVuWGFBVjY0UUlKem5jTG5SLWJ5UV9EV05vUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>OneSoil is in the news for its AI Agronomist tool, which provides actionable advice to farmers by analyzing fragmented farm data.</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>2026-06-22 14:32:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>AeroFarms</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Not Mentioned</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Vertical Farming</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>AeroFarms is a vertical farming company known for growing produce indoors using aeroponics technology.</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Acquisition</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxObFRmQUxNTTFhVkZLY005S2V2UnZGWkJvQVl1MkMzU3lkWHg0ZzVyaU9XbkswdHlOaFEtOF9CWHRlUXo1VHhVTElOMkFPQ3pVd2lzNlpTSXNFZmVBMjhPeU1GTnZaNkhIeEJJbTBIc3EtcURQcjZBdmNTckg4dnN1dy1Sal94NVBlb2hlak5CQXNzMU5uQkVCaTBRM055Y2IzVGR2OEUtc3c2aEg0SFJjWkdzZzhvYkljLVBCdUtNLXRZbmkxcTdabA?oc=5</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>AeroFarms, a vertical farming company, was acquired.</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>2026-06-22 14:33:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Seqana</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Not Mentioned</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Seqana is a SaaS company, but the specific details of its core technology or product within the AgTech sector are not provided in the snippet.</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>€3.2M</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Funding</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiakFVX3lxTE5naEZsUXhDTmp3SW9ud1FTcHJ0RjhqZ2hNMGJxaHY1SWZ0ZTl2Um5hdFcxTXVMNjR4ZjdwRm56djFrc1FiRVRrYnVINm5vakRkeVFSNnRUVG14OWpGTE5JQ0lRQnZvaWp1VHc?oc=5</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Seqana secured €3.2M in funding.</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>2026-06-22 14:33:35</t>
         </is>
       </c>
     </row>

</xml_diff>